<commit_message>
fix: apply weslh translations to multi year
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/multi-year/xlsx/02-account-home-manage-recycling-obligations-tile.xlsx
+++ b/translations/welsh-translations/multi-year/xlsx/02-account-home-manage-recycling-obligations-tile.xlsx
@@ -93,7 +93,7 @@
     <t>An approved or delegated person must submit your {0} certificate of compliance on or before {1:d MMMM yyyy}.</t>
   </si>
   <si>
-    <t>Rhaid i berson wedi’i gymeradwyo neu wedi’i ddirprwyo gyflwyno’ch tystysgrif gydymffurfio {0} ar neu cyn {1:d MMMM bbbb}.</t>
+    <t>Rhaid i berson wedi’i gymeradwyo neu wedi’i ddirprwyo gyflwyno’ch tystysgrif gydymffurfio {0} ar neu cyn {1:d MMMM yyyy}.</t>
   </si>
   <si>
     <t>src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTileMultiYear.en.resx::submit_compliance_by_deadline_compliance_scheme</t>
@@ -105,7 +105,7 @@
     <t>An approved or delegated person must submit your {0} statement of compliance on or before {1:d MMMM yyyy}.</t>
   </si>
   <si>
-    <t>Rhaid i berson wedi’i gymeradwyo neu wedi’i ddirprwyo gyflwyno'ch datganiad cydymffurfio {0} ar neu cyn {1:d MMMM bbbb}.</t>
+    <t>Rhaid i berson wedi’i gymeradwyo neu wedi’i ddirprwyo gyflwyno'ch datganiad cydymffurfio {0} ar neu cyn {1:d MMMM yyyy}.</t>
   </si>
   <si>
     <t>src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTileMultiYear.en.resx::search_all_link</t>

</xml_diff>